<commit_message>
Integrate exact-tied eQTL variants
</commit_message>
<xml_diff>
--- a/processed-data/11_eQTL_coloc/seurat/final/coloc_results.xlsx
+++ b/processed-data/11_eQTL_coloc/seurat/final/coloc_results.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="300">
   <si>
     <t xml:space="preserve">disorder</t>
   </si>
@@ -874,9 +874,6 @@
   </si>
   <si>
     <t xml:space="preserve">AP001505.1, FADS1, NTSR1, VWA5B2, WAC-AS1</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
   </si>
   <si>
     <t xml:space="preserve">FBLN7, SPSB2, TMEM258</t>
@@ -1502,7 +1499,7 @@
         <v>0</v>
       </c>
       <c r="U2" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" s="5" t="n">
         <v>1</v>
@@ -1668,7 +1665,7 @@
         <v>1</v>
       </c>
       <c r="U4" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V4" s="5" t="n">
         <v>1</v>
@@ -2498,7 +2495,7 @@
         <v>0</v>
       </c>
       <c r="U14" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" s="5" t="n">
         <v>1</v>
@@ -2913,7 +2910,7 @@
         <v>1</v>
       </c>
       <c r="U19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V19" s="5" t="n">
         <v>1</v>
@@ -3328,7 +3325,7 @@
         <v>0</v>
       </c>
       <c r="U24" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V24" s="5" t="n">
         <v>1</v>
@@ -3411,7 +3408,7 @@
         <v>0</v>
       </c>
       <c r="U25" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V25" s="5" t="n">
         <v>1</v>
@@ -3577,7 +3574,7 @@
         <v>1</v>
       </c>
       <c r="U27" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V27" s="5" t="n">
         <v>1</v>
@@ -3660,7 +3657,7 @@
         <v>0</v>
       </c>
       <c r="U28" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V28" s="5" t="n">
         <v>1</v>
@@ -3909,7 +3906,7 @@
         <v>0</v>
       </c>
       <c r="U31" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V31" s="5" t="n">
         <v>1</v>
@@ -4241,7 +4238,7 @@
         <v>0</v>
       </c>
       <c r="U35" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V35" s="5" t="n">
         <v>1</v>
@@ -6960,7 +6957,7 @@
         <v>0</v>
       </c>
       <c r="U68" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V68" s="5" t="n">
         <v>1</v>
@@ -9762,9 +9759,7 @@
       <c r="E8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="s">
-        <v>287</v>
-      </c>
+      <c r="F8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
@@ -9803,7 +9798,7 @@
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11">
@@ -9823,7 +9818,7 @@
         <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="12">
@@ -9843,7 +9838,7 @@
         <v>7</v>
       </c>
       <c r="F12" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="13">
@@ -9863,7 +9858,7 @@
         <v>3</v>
       </c>
       <c r="F13" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="14">
@@ -9883,7 +9878,7 @@
         <v>5</v>
       </c>
       <c r="F14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="15">
@@ -9903,7 +9898,7 @@
         <v>2</v>
       </c>
       <c r="F15" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="16">
@@ -9943,7 +9938,7 @@
         <v>2</v>
       </c>
       <c r="F17" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="18">
@@ -9963,7 +9958,7 @@
         <v>5</v>
       </c>
       <c r="F18" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="19">
@@ -9983,7 +9978,7 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="20">
@@ -10003,7 +9998,7 @@
         <v>9</v>
       </c>
       <c r="F20" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="21">
@@ -10023,7 +10018,7 @@
         <v>6</v>
       </c>
       <c r="F21" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="22">
@@ -10043,7 +10038,7 @@
         <v>6</v>
       </c>
       <c r="F22" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="23">
@@ -10063,7 +10058,7 @@
         <v>7</v>
       </c>
       <c r="F23" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Correct DEG annotations to authoritative 503-gene set
</commit_message>
<xml_diff>
--- a/processed-data/11_eQTL_coloc/seurat/final/coloc_results.xlsx
+++ b/processed-data/11_eQTL_coloc/seurat/final/coloc_results.xlsx
@@ -6948,7 +6948,7 @@
         <v>3</v>
       </c>
       <c r="R68" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S68" s="5" t="n">
         <v>0</v>
@@ -7264,7 +7264,7 @@
         <v>4</v>
       </c>
       <c r="R72" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S72" s="5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Mark unavailable SCZD exploratory support as N/A in ST7
Display missing SCZD exploratory flags as literal N/A in both workbook export paths while preserving analytical missing values. Treat N/A as missing in workbook readers to retain numeric GWAS flags and existing variant counts. Include the regenerated ST7 workbook; only Z63:AA101 changes.
</commit_message>
<xml_diff>
--- a/processed-data/11_eQTL_coloc/seurat/final/coloc_results.xlsx
+++ b/processed-data/11_eQTL_coloc/seurat/final/coloc_results.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="301">
   <si>
     <t xml:space="preserve">disorder</t>
   </si>
@@ -847,6 +847,9 @@
   </si>
   <si>
     <t xml:space="preserve">rs2189336</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A</t>
   </si>
   <si>
     <t xml:space="preserve">n_tested_genes</t>
@@ -6576,8 +6579,12 @@
       <c r="Y63" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z63" s="5"/>
-      <c r="AA63" s="5"/>
+      <c r="Z63" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA63" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
@@ -6655,8 +6662,12 @@
       <c r="Y64" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z64" s="5"/>
-      <c r="AA64" s="5"/>
+      <c r="Z64" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA64" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
@@ -6734,8 +6745,12 @@
       <c r="Y65" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z65" s="5"/>
-      <c r="AA65" s="5"/>
+      <c r="Z65" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA65" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
@@ -6813,8 +6828,12 @@
       <c r="Y66" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z66" s="5"/>
-      <c r="AA66" s="5"/>
+      <c r="Z66" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA66" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
@@ -6892,8 +6911,12 @@
       <c r="Y67" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z67" s="5"/>
-      <c r="AA67" s="5"/>
+      <c r="Z67" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA67" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
@@ -6971,8 +6994,12 @@
       <c r="Y68" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z68" s="5"/>
-      <c r="AA68" s="5"/>
+      <c r="Z68" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA68" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
@@ -7050,8 +7077,12 @@
       <c r="Y69" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z69" s="5"/>
-      <c r="AA69" s="5"/>
+      <c r="Z69" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA69" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
@@ -7129,8 +7160,12 @@
       <c r="Y70" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z70" s="5"/>
-      <c r="AA70" s="5"/>
+      <c r="Z70" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA70" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
@@ -7208,8 +7243,12 @@
       <c r="Y71" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z71" s="5"/>
-      <c r="AA71" s="5"/>
+      <c r="Z71" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA71" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
@@ -7287,8 +7326,12 @@
       <c r="Y72" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z72" s="5"/>
-      <c r="AA72" s="5"/>
+      <c r="Z72" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA72" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
@@ -7366,8 +7409,12 @@
       <c r="Y73" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z73" s="5"/>
-      <c r="AA73" s="5"/>
+      <c r="Z73" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA73" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
@@ -7445,8 +7492,12 @@
       <c r="Y74" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z74" s="5"/>
-      <c r="AA74" s="5"/>
+      <c r="Z74" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA74" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
@@ -7524,8 +7575,12 @@
       <c r="Y75" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z75" s="5"/>
-      <c r="AA75" s="5"/>
+      <c r="Z75" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA75" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
@@ -7603,8 +7658,12 @@
       <c r="Y76" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z76" s="5"/>
-      <c r="AA76" s="5"/>
+      <c r="Z76" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA76" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
@@ -7682,8 +7741,12 @@
       <c r="Y77" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z77" s="5"/>
-      <c r="AA77" s="5"/>
+      <c r="Z77" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA77" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
@@ -7761,8 +7824,12 @@
       <c r="Y78" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z78" s="5"/>
-      <c r="AA78" s="5"/>
+      <c r="Z78" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA78" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
@@ -7840,8 +7907,12 @@
       <c r="Y79" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z79" s="5"/>
-      <c r="AA79" s="5"/>
+      <c r="Z79" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA79" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="s">
@@ -7919,8 +7990,12 @@
       <c r="Y80" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z80" s="5"/>
-      <c r="AA80" s="5"/>
+      <c r="Z80" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA80" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
@@ -7998,8 +8073,12 @@
       <c r="Y81" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z81" s="5"/>
-      <c r="AA81" s="5"/>
+      <c r="Z81" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA81" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
@@ -8077,8 +8156,12 @@
       <c r="Y82" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z82" s="5"/>
-      <c r="AA82" s="5"/>
+      <c r="Z82" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA82" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="s">
@@ -8156,8 +8239,12 @@
       <c r="Y83" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z83" s="5"/>
-      <c r="AA83" s="5"/>
+      <c r="Z83" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA83" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
@@ -8235,8 +8322,12 @@
       <c r="Y84" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z84" s="5"/>
-      <c r="AA84" s="5"/>
+      <c r="Z84" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA84" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="s">
@@ -8314,8 +8405,12 @@
       <c r="Y85" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z85" s="5"/>
-      <c r="AA85" s="5"/>
+      <c r="Z85" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA85" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
@@ -8393,8 +8488,12 @@
       <c r="Y86" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z86" s="5"/>
-      <c r="AA86" s="5"/>
+      <c r="Z86" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA86" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
@@ -8472,8 +8571,12 @@
       <c r="Y87" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z87" s="5"/>
-      <c r="AA87" s="5"/>
+      <c r="Z87" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA87" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
@@ -8551,8 +8654,12 @@
       <c r="Y88" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z88" s="5"/>
-      <c r="AA88" s="5"/>
+      <c r="Z88" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA88" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
@@ -8630,8 +8737,12 @@
       <c r="Y89" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z89" s="5"/>
-      <c r="AA89" s="5"/>
+      <c r="Z89" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA89" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
@@ -8709,8 +8820,12 @@
       <c r="Y90" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z90" s="5"/>
-      <c r="AA90" s="5"/>
+      <c r="Z90" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA90" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
@@ -8788,8 +8903,12 @@
       <c r="Y91" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z91" s="5"/>
-      <c r="AA91" s="5"/>
+      <c r="Z91" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA91" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
@@ -8867,8 +8986,12 @@
       <c r="Y92" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z92" s="5"/>
-      <c r="AA92" s="5"/>
+      <c r="Z92" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA92" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
@@ -8946,8 +9069,12 @@
       <c r="Y93" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z93" s="5"/>
-      <c r="AA93" s="5"/>
+      <c r="Z93" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA93" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="s">
@@ -9025,8 +9152,12 @@
       <c r="Y94" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z94" s="5"/>
-      <c r="AA94" s="5"/>
+      <c r="Z94" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA94" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="s">
@@ -9104,8 +9235,12 @@
       <c r="Y95" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z95" s="5"/>
-      <c r="AA95" s="5"/>
+      <c r="Z95" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA95" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="s">
@@ -9183,8 +9318,12 @@
       <c r="Y96" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="Z96" s="5"/>
-      <c r="AA96" s="5"/>
+      <c r="Z96" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA96" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="s">
@@ -9262,8 +9401,12 @@
       <c r="Y97" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z97" s="5"/>
-      <c r="AA97" s="5"/>
+      <c r="Z97" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA97" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="s">
@@ -9341,8 +9484,12 @@
       <c r="Y98" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z98" s="5"/>
-      <c r="AA98" s="5"/>
+      <c r="Z98" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA98" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="s">
@@ -9420,8 +9567,12 @@
       <c r="Y99" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z99" s="5"/>
-      <c r="AA99" s="5"/>
+      <c r="Z99" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA99" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="s">
@@ -9499,8 +9650,12 @@
       <c r="Y100" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z100" s="5"/>
-      <c r="AA100" s="5"/>
+      <c r="Z100" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA100" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
@@ -9578,8 +9733,12 @@
       <c r="Y101" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="Z101" s="5"/>
-      <c r="AA101" s="5"/>
+      <c r="Z101" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA101" s="5" t="s">
+        <v>278</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9611,16 +9770,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2">
@@ -9640,7 +9799,7 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3">
@@ -9660,7 +9819,7 @@
         <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4">
@@ -9680,7 +9839,7 @@
         <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5">
@@ -9720,7 +9879,7 @@
         <v>7</v>
       </c>
       <c r="F6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7">
@@ -9740,7 +9899,7 @@
         <v>5</v>
       </c>
       <c r="F7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="8">
@@ -9798,7 +9957,7 @@
         <v>3</v>
       </c>
       <c r="F10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11">
@@ -9818,7 +9977,7 @@
         <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="12">
@@ -9838,7 +9997,7 @@
         <v>7</v>
       </c>
       <c r="F12" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="13">
@@ -9858,7 +10017,7 @@
         <v>3</v>
       </c>
       <c r="F13" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="14">
@@ -9878,7 +10037,7 @@
         <v>5</v>
       </c>
       <c r="F14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="15">
@@ -9898,7 +10057,7 @@
         <v>2</v>
       </c>
       <c r="F15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="16">
@@ -9938,7 +10097,7 @@
         <v>2</v>
       </c>
       <c r="F17" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="18">
@@ -9958,7 +10117,7 @@
         <v>5</v>
       </c>
       <c r="F18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="19">
@@ -9978,7 +10137,7 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="20">
@@ -9998,7 +10157,7 @@
         <v>9</v>
       </c>
       <c r="F20" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="21">
@@ -10018,7 +10177,7 @@
         <v>6</v>
       </c>
       <c r="F21" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="22">
@@ -10038,7 +10197,7 @@
         <v>6</v>
       </c>
       <c r="F22" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="23">
@@ -10058,7 +10217,7 @@
         <v>7</v>
       </c>
       <c r="F23" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="24">

</xml_diff>